<commit_message>
fix: update sample excel file
</commit_message>
<xml_diff>
--- a/frontend/sample_files/_SoIT Lecture and  Tutor List Sem1 2026- For SETU.xlsx
+++ b/frontend/sample_files/_SoIT Lecture and  Tutor List Sem1 2026- For SETU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yychuah/Documents/docs/YEAR 3/FYP/FYPMCS07/frontend/sample_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9153E48-3376-BF47-82FE-B80FDF3D666E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E33DC0CD-BC2C-6A48-959A-0DF8EC54DF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1767,18 +1767,36 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1787,43 +1805,10 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1840,7 +1825,22 @@
     <xf numFmtId="49" fontId="6" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2201,50 +2201,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="13">
-      <c r="A1" s="76"/>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="77" t="s">
+      <c r="A1" s="71"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
     </row>
     <row r="2" spans="1:10" ht="13">
-      <c r="A2" s="78" t="s">
+      <c r="A2" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="78" t="s">
+      <c r="B2" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="78" t="s">
+      <c r="C2" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="78" t="s">
+      <c r="D2" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="64" t="s">
+      <c r="E2" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="65"/>
-      <c r="G2" s="64" t="s">
+      <c r="F2" s="55"/>
+      <c r="G2" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="65"/>
-      <c r="I2" s="64" t="s">
+      <c r="H2" s="55"/>
+      <c r="I2" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="65"/>
+      <c r="J2" s="55"/>
     </row>
     <row r="3" spans="1:10" ht="15">
-      <c r="A3" s="48"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
+      <c r="A3" s="47"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
       <c r="E3" s="3" t="s">
         <v>16</v>
       </c>
@@ -2265,16 +2265,16 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="15">
-      <c r="A4" s="46">
+      <c r="A4" s="61">
         <v>1</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="52" t="s">
+      <c r="D4" s="64" t="s">
         <v>22</v>
       </c>
       <c r="E4" s="5" t="s">
@@ -2289,20 +2289,20 @@
       <c r="H4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="66" t="s">
+      <c r="I4" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="67"/>
+      <c r="J4" s="50"/>
     </row>
     <row r="5" spans="1:10" ht="15">
-      <c r="A5" s="47"/>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="51" t="s">
+      <c r="A5" s="60"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="F5" s="51" t="s">
+      <c r="F5" s="46" t="s">
         <v>42</v>
       </c>
       <c r="G5" s="5" t="s">
@@ -2311,72 +2311,72 @@
       <c r="H5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="I5" s="61"/>
-      <c r="J5" s="68"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="58"/>
     </row>
     <row r="6" spans="1:10" ht="15">
-      <c r="A6" s="47"/>
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
+      <c r="A6" s="60"/>
+      <c r="B6" s="60"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
       <c r="G6" s="5" t="s">
         <v>43</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="61"/>
-      <c r="J6" s="68"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="58"/>
     </row>
     <row r="7" spans="1:10" ht="15">
-      <c r="A7" s="47"/>
-      <c r="B7" s="47"/>
-      <c r="C7" s="47"/>
-      <c r="D7" s="47"/>
-      <c r="E7" s="47"/>
-      <c r="F7" s="47"/>
+      <c r="A7" s="60"/>
+      <c r="B7" s="60"/>
+      <c r="C7" s="60"/>
+      <c r="D7" s="60"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="60"/>
       <c r="G7" s="5" t="s">
         <v>47</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="61"/>
-      <c r="J7" s="68"/>
+      <c r="I7" s="56"/>
+      <c r="J7" s="58"/>
     </row>
     <row r="8" spans="1:10" ht="15">
-      <c r="A8" s="47"/>
-      <c r="B8" s="47"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="47"/>
-      <c r="F8" s="47"/>
+      <c r="A8" s="60"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="60"/>
       <c r="G8" s="5" t="s">
         <v>49</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="I8" s="61"/>
-      <c r="J8" s="68"/>
+      <c r="I8" s="56"/>
+      <c r="J8" s="58"/>
     </row>
     <row r="9" spans="1:10" ht="15">
-      <c r="A9" s="48"/>
-      <c r="B9" s="48"/>
-      <c r="C9" s="48"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="47"/>
-      <c r="F9" s="47"/>
+      <c r="A9" s="47"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="60"/>
       <c r="G9" s="5" t="s">
         <v>51</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I9" s="61"/>
-      <c r="J9" s="68"/>
+      <c r="I9" s="56"/>
+      <c r="J9" s="58"/>
     </row>
     <row r="10" spans="1:10" ht="30">
       <c r="A10" s="8">
@@ -2391,34 +2391,34 @@
       <c r="D10" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
       <c r="G10" s="5" t="s">
         <v>60</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="I10" s="61"/>
-      <c r="J10" s="68"/>
+      <c r="I10" s="56"/>
+      <c r="J10" s="58"/>
     </row>
     <row r="11" spans="1:10" ht="15">
-      <c r="A11" s="46">
+      <c r="A11" s="61">
         <v>3</v>
       </c>
-      <c r="B11" s="46" t="s">
+      <c r="B11" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="61" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="52" t="s">
+      <c r="D11" s="64" t="s">
         <v>65</v>
       </c>
-      <c r="E11" s="51" t="s">
+      <c r="E11" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="51" t="s">
+      <c r="F11" s="46" t="s">
         <v>68</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -2427,140 +2427,140 @@
       <c r="H11" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="I11" s="61"/>
-      <c r="J11" s="68"/>
+      <c r="I11" s="56"/>
+      <c r="J11" s="58"/>
     </row>
     <row r="12" spans="1:10" ht="15">
-      <c r="A12" s="48"/>
-      <c r="B12" s="48"/>
-      <c r="C12" s="48"/>
-      <c r="D12" s="48"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="47"/>
+      <c r="A12" s="47"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
       <c r="G12" s="5" t="s">
         <v>74</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="I12" s="61"/>
-      <c r="J12" s="68"/>
+      <c r="I12" s="56"/>
+      <c r="J12" s="58"/>
     </row>
     <row r="13" spans="1:10" ht="15">
-      <c r="A13" s="46">
+      <c r="A13" s="61">
         <v>4</v>
       </c>
-      <c r="B13" s="46" t="s">
+      <c r="B13" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="46" t="s">
+      <c r="C13" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="D13" s="52" t="s">
+      <c r="D13" s="64" t="s">
         <v>83</v>
       </c>
-      <c r="E13" s="66"/>
-      <c r="F13" s="67"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="50"/>
       <c r="G13" s="11" t="s">
         <v>39</v>
       </c>
       <c r="H13" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="I13" s="61"/>
-      <c r="J13" s="68"/>
+      <c r="I13" s="56"/>
+      <c r="J13" s="58"/>
     </row>
     <row r="14" spans="1:10" ht="15">
-      <c r="A14" s="47"/>
-      <c r="B14" s="47"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="61"/>
-      <c r="F14" s="68"/>
+      <c r="A14" s="60"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="60"/>
+      <c r="D14" s="60"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="58"/>
       <c r="G14" s="5" t="s">
         <v>84</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="61"/>
-      <c r="J14" s="68"/>
+      <c r="I14" s="56"/>
+      <c r="J14" s="58"/>
     </row>
     <row r="15" spans="1:10" ht="15">
-      <c r="A15" s="47"/>
-      <c r="B15" s="47"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="47"/>
-      <c r="E15" s="61"/>
-      <c r="F15" s="68"/>
+      <c r="A15" s="60"/>
+      <c r="B15" s="60"/>
+      <c r="C15" s="60"/>
+      <c r="D15" s="60"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="58"/>
       <c r="G15" s="5" t="s">
         <v>88</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="I15" s="61"/>
-      <c r="J15" s="68"/>
+      <c r="I15" s="56"/>
+      <c r="J15" s="58"/>
     </row>
     <row r="16" spans="1:10" ht="15">
-      <c r="A16" s="47"/>
-      <c r="B16" s="47"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="61"/>
-      <c r="F16" s="68"/>
+      <c r="A16" s="60"/>
+      <c r="B16" s="60"/>
+      <c r="C16" s="60"/>
+      <c r="D16" s="60"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="58"/>
       <c r="G16" s="5" t="s">
         <v>90</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="I16" s="61"/>
-      <c r="J16" s="68"/>
+      <c r="I16" s="56"/>
+      <c r="J16" s="58"/>
     </row>
     <row r="17" spans="1:10" ht="15">
-      <c r="A17" s="47"/>
-      <c r="B17" s="47"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="68"/>
+      <c r="A17" s="60"/>
+      <c r="B17" s="60"/>
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="58"/>
       <c r="G17" s="5" t="s">
         <v>93</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="I17" s="61"/>
-      <c r="J17" s="68"/>
+      <c r="I17" s="56"/>
+      <c r="J17" s="58"/>
     </row>
     <row r="18" spans="1:10" ht="15">
-      <c r="A18" s="48"/>
-      <c r="B18" s="48"/>
-      <c r="C18" s="48"/>
-      <c r="D18" s="48"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="68"/>
+      <c r="A18" s="47"/>
+      <c r="B18" s="47"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="58"/>
       <c r="G18" s="5" t="s">
         <v>96</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="I18" s="61"/>
-      <c r="J18" s="68"/>
+      <c r="I18" s="56"/>
+      <c r="J18" s="58"/>
     </row>
     <row r="19" spans="1:10" ht="15">
-      <c r="A19" s="46">
+      <c r="A19" s="61">
         <v>5</v>
       </c>
-      <c r="B19" s="49" t="s">
+      <c r="B19" s="62" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="49" t="s">
+      <c r="C19" s="62" t="s">
         <v>101</v>
       </c>
-      <c r="D19" s="50" t="s">
+      <c r="D19" s="63" t="s">
         <v>104</v>
       </c>
       <c r="E19" s="11" t="s">
@@ -2575,18 +2575,18 @@
       <c r="H19" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="I19" s="61"/>
-      <c r="J19" s="68"/>
+      <c r="I19" s="56"/>
+      <c r="J19" s="58"/>
     </row>
     <row r="20" spans="1:10" ht="24.75" customHeight="1">
-      <c r="A20" s="48"/>
-      <c r="B20" s="47"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="56" t="s">
+      <c r="A20" s="47"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="60"/>
+      <c r="D20" s="60"/>
+      <c r="E20" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="F20" s="56" t="s">
+      <c r="F20" s="59" t="s">
         <v>109</v>
       </c>
       <c r="G20" s="6" t="s">
@@ -2595,36 +2595,36 @@
       <c r="H20" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="I20" s="61"/>
-      <c r="J20" s="68"/>
+      <c r="I20" s="56"/>
+      <c r="J20" s="58"/>
     </row>
     <row r="21" spans="1:10" ht="24.75" customHeight="1">
       <c r="A21" s="8"/>
-      <c r="B21" s="48"/>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
+      <c r="B21" s="47"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="47"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="47"/>
       <c r="G21" s="6" t="s">
         <v>117</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="I21" s="61"/>
-      <c r="J21" s="68"/>
+      <c r="I21" s="56"/>
+      <c r="J21" s="58"/>
     </row>
     <row r="22" spans="1:10" ht="15">
-      <c r="A22" s="46">
+      <c r="A22" s="61">
         <v>6</v>
       </c>
-      <c r="B22" s="49" t="s">
+      <c r="B22" s="62" t="s">
         <v>98</v>
       </c>
-      <c r="C22" s="49" t="s">
+      <c r="C22" s="62" t="s">
         <v>121</v>
       </c>
-      <c r="D22" s="50" t="s">
+      <c r="D22" s="63" t="s">
         <v>123</v>
       </c>
       <c r="E22" s="11" t="s">
@@ -2639,18 +2639,18 @@
       <c r="H22" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="I22" s="61"/>
-      <c r="J22" s="68"/>
+      <c r="I22" s="56"/>
+      <c r="J22" s="58"/>
     </row>
     <row r="23" spans="1:10" ht="15">
-      <c r="A23" s="47"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="51" t="s">
+      <c r="A23" s="60"/>
+      <c r="B23" s="60"/>
+      <c r="C23" s="60"/>
+      <c r="D23" s="60"/>
+      <c r="E23" s="46" t="s">
         <v>132</v>
       </c>
-      <c r="F23" s="51" t="s">
+      <c r="F23" s="46" t="s">
         <v>133</v>
       </c>
       <c r="G23" s="6" t="s">
@@ -2659,52 +2659,52 @@
       <c r="H23" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="I23" s="61"/>
-      <c r="J23" s="68"/>
+      <c r="I23" s="56"/>
+      <c r="J23" s="58"/>
     </row>
     <row r="24" spans="1:10" ht="15">
-      <c r="A24" s="47"/>
-      <c r="B24" s="47"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="47"/>
+      <c r="A24" s="60"/>
+      <c r="B24" s="60"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="60"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="60"/>
       <c r="G24" s="6" t="s">
         <v>33</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="I24" s="61"/>
-      <c r="J24" s="68"/>
+      <c r="I24" s="56"/>
+      <c r="J24" s="58"/>
     </row>
     <row r="25" spans="1:10" ht="15">
-      <c r="A25" s="48"/>
-      <c r="B25" s="48"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="48"/>
+      <c r="A25" s="47"/>
+      <c r="B25" s="47"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="47"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="47"/>
       <c r="G25" s="6" t="s">
         <v>144</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="I25" s="61"/>
-      <c r="J25" s="68"/>
+      <c r="I25" s="56"/>
+      <c r="J25" s="58"/>
     </row>
     <row r="26" spans="1:10" ht="15">
-      <c r="A26" s="46">
+      <c r="A26" s="61">
         <v>7</v>
       </c>
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="46" t="s">
+      <c r="C26" s="61" t="s">
         <v>152</v>
       </c>
-      <c r="D26" s="52" t="s">
+      <c r="D26" s="64" t="s">
         <v>153</v>
       </c>
       <c r="E26" s="11" t="s">
@@ -2719,18 +2719,18 @@
       <c r="H26" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="I26" s="61"/>
-      <c r="J26" s="68"/>
+      <c r="I26" s="56"/>
+      <c r="J26" s="58"/>
     </row>
     <row r="27" spans="1:10" ht="15">
-      <c r="A27" s="47"/>
-      <c r="B27" s="47"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="51" t="s">
+      <c r="A27" s="60"/>
+      <c r="B27" s="60"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="60"/>
+      <c r="E27" s="46" t="s">
         <v>135</v>
       </c>
-      <c r="F27" s="51" t="s">
+      <c r="F27" s="46" t="s">
         <v>134</v>
       </c>
       <c r="G27" s="5" t="s">
@@ -2739,36 +2739,36 @@
       <c r="H27" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="I27" s="61"/>
-      <c r="J27" s="68"/>
+      <c r="I27" s="56"/>
+      <c r="J27" s="58"/>
     </row>
     <row r="28" spans="1:10" ht="15">
-      <c r="A28" s="48"/>
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="48"/>
+      <c r="A28" s="47"/>
+      <c r="B28" s="47"/>
+      <c r="C28" s="47"/>
+      <c r="D28" s="47"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="47"/>
       <c r="G28" s="5" t="s">
         <v>88</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="I28" s="61"/>
-      <c r="J28" s="68"/>
+      <c r="I28" s="56"/>
+      <c r="J28" s="58"/>
     </row>
     <row r="29" spans="1:10" ht="15">
-      <c r="A29" s="46">
+      <c r="A29" s="61">
         <v>8</v>
       </c>
-      <c r="B29" s="49" t="s">
+      <c r="B29" s="62" t="s">
         <v>98</v>
       </c>
-      <c r="C29" s="49" t="s">
+      <c r="C29" s="62" t="s">
         <v>173</v>
       </c>
-      <c r="D29" s="50" t="s">
+      <c r="D29" s="63" t="s">
         <v>174</v>
       </c>
       <c r="E29" s="16" t="s">
@@ -2783,14 +2783,14 @@
       <c r="H29" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="I29" s="61"/>
-      <c r="J29" s="68"/>
+      <c r="I29" s="56"/>
+      <c r="J29" s="58"/>
     </row>
     <row r="30" spans="1:10" ht="26.25" customHeight="1">
-      <c r="A30" s="47"/>
-      <c r="B30" s="47"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
+      <c r="A30" s="60"/>
+      <c r="B30" s="60"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="60"/>
       <c r="E30" s="16" t="s">
         <v>177</v>
       </c>
@@ -2803,14 +2803,14 @@
       <c r="H30" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="I30" s="61"/>
-      <c r="J30" s="68"/>
+      <c r="I30" s="56"/>
+      <c r="J30" s="58"/>
     </row>
     <row r="31" spans="1:10" ht="26.25" customHeight="1">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
+      <c r="A31" s="47"/>
+      <c r="B31" s="47"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="47"/>
       <c r="E31" s="6" t="s">
         <v>181</v>
       </c>
@@ -2823,26 +2823,26 @@
       <c r="H31" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="I31" s="61"/>
-      <c r="J31" s="68"/>
+      <c r="I31" s="56"/>
+      <c r="J31" s="58"/>
     </row>
     <row r="32" spans="1:10" ht="15">
-      <c r="A32" s="46">
+      <c r="A32" s="61">
         <v>9</v>
       </c>
-      <c r="B32" s="46" t="s">
+      <c r="B32" s="61" t="s">
         <v>55</v>
       </c>
-      <c r="C32" s="46" t="s">
+      <c r="C32" s="61" t="s">
         <v>187</v>
       </c>
-      <c r="D32" s="53" t="s">
+      <c r="D32" s="65" t="s">
         <v>190</v>
       </c>
-      <c r="E32" s="51" t="s">
+      <c r="E32" s="46" t="s">
         <v>175</v>
       </c>
-      <c r="F32" s="51" t="s">
+      <c r="F32" s="46" t="s">
         <v>176</v>
       </c>
       <c r="G32" s="6" t="s">
@@ -2851,42 +2851,42 @@
       <c r="H32" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="I32" s="61"/>
-      <c r="J32" s="68"/>
+      <c r="I32" s="56"/>
+      <c r="J32" s="58"/>
     </row>
     <row r="33" spans="1:10" ht="15">
-      <c r="A33" s="54"/>
-      <c r="B33" s="54"/>
-      <c r="C33" s="54"/>
-      <c r="D33" s="54"/>
-      <c r="E33" s="54"/>
-      <c r="F33" s="54"/>
+      <c r="A33" s="79"/>
+      <c r="B33" s="79"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="79"/>
+      <c r="E33" s="79"/>
+      <c r="F33" s="79"/>
       <c r="G33" s="31" t="s">
         <v>117</v>
       </c>
       <c r="H33" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="I33" s="61"/>
-      <c r="J33" s="68"/>
+      <c r="I33" s="56"/>
+      <c r="J33" s="58"/>
     </row>
     <row r="34" spans="1:10" ht="15">
-      <c r="A34" s="57">
+      <c r="A34" s="66">
         <v>10</v>
       </c>
-      <c r="B34" s="58" t="s">
+      <c r="B34" s="75" t="s">
         <v>98</v>
       </c>
-      <c r="C34" s="58" t="s">
+      <c r="C34" s="75" t="s">
         <v>206</v>
       </c>
-      <c r="D34" s="59" t="s">
+      <c r="D34" s="76" t="s">
         <v>210</v>
       </c>
-      <c r="E34" s="55" t="s">
+      <c r="E34" s="74" t="s">
         <v>53</v>
       </c>
-      <c r="F34" s="60" t="s">
+      <c r="F34" s="77" t="s">
         <v>136</v>
       </c>
       <c r="G34" s="32" t="s">
@@ -2895,90 +2895,90 @@
       <c r="H34" s="32" t="s">
         <v>136</v>
       </c>
-      <c r="I34" s="61"/>
-      <c r="J34" s="68"/>
+      <c r="I34" s="56"/>
+      <c r="J34" s="58"/>
     </row>
     <row r="35" spans="1:10" ht="15" hidden="1">
-      <c r="A35" s="47"/>
-      <c r="B35" s="47"/>
-      <c r="C35" s="47"/>
-      <c r="D35" s="47"/>
-      <c r="E35" s="47"/>
-      <c r="F35" s="61"/>
+      <c r="A35" s="60"/>
+      <c r="B35" s="60"/>
+      <c r="C35" s="60"/>
+      <c r="D35" s="60"/>
+      <c r="E35" s="60"/>
+      <c r="F35" s="56"/>
       <c r="G35" s="5" t="s">
         <v>222</v>
       </c>
       <c r="H35" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="I35" s="61"/>
-      <c r="J35" s="68"/>
+      <c r="I35" s="56"/>
+      <c r="J35" s="58"/>
     </row>
     <row r="36" spans="1:10" ht="15">
-      <c r="A36" s="47"/>
-      <c r="B36" s="47"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="47"/>
-      <c r="E36" s="47"/>
-      <c r="F36" s="61"/>
+      <c r="A36" s="60"/>
+      <c r="B36" s="60"/>
+      <c r="C36" s="60"/>
+      <c r="D36" s="60"/>
+      <c r="E36" s="60"/>
+      <c r="F36" s="56"/>
       <c r="G36" s="5" t="s">
         <v>228</v>
       </c>
       <c r="H36" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="I36" s="61"/>
-      <c r="J36" s="68"/>
+      <c r="I36" s="56"/>
+      <c r="J36" s="58"/>
     </row>
     <row r="37" spans="1:10" ht="15" hidden="1">
-      <c r="A37" s="47"/>
-      <c r="B37" s="47"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="47"/>
-      <c r="E37" s="47"/>
-      <c r="F37" s="61"/>
+      <c r="A37" s="60"/>
+      <c r="B37" s="60"/>
+      <c r="C37" s="60"/>
+      <c r="D37" s="60"/>
+      <c r="E37" s="60"/>
+      <c r="F37" s="56"/>
       <c r="G37" s="5" t="s">
         <v>40</v>
       </c>
       <c r="H37" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="I37" s="61"/>
-      <c r="J37" s="68"/>
+      <c r="I37" s="56"/>
+      <c r="J37" s="58"/>
     </row>
     <row r="38" spans="1:10" ht="15">
-      <c r="A38" s="48"/>
-      <c r="B38" s="48"/>
-      <c r="C38" s="48"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="47"/>
-      <c r="F38" s="61"/>
+      <c r="A38" s="47"/>
+      <c r="B38" s="47"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="47"/>
+      <c r="E38" s="60"/>
+      <c r="F38" s="56"/>
       <c r="G38" s="5" t="s">
         <v>241</v>
       </c>
       <c r="H38" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="I38" s="61"/>
-      <c r="J38" s="68"/>
+      <c r="I38" s="56"/>
+      <c r="J38" s="58"/>
     </row>
     <row r="39" spans="1:10" ht="15">
-      <c r="A39" s="46">
+      <c r="A39" s="61">
         <v>11</v>
       </c>
-      <c r="B39" s="46" t="s">
+      <c r="B39" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C39" s="46" t="s">
+      <c r="C39" s="61" t="s">
         <v>244</v>
       </c>
-      <c r="D39" s="62" t="s">
+      <c r="D39" s="78" t="s">
         <v>245</v>
       </c>
-      <c r="E39" s="56" t="s">
+      <c r="E39" s="59" t="s">
         <v>222</v>
       </c>
-      <c r="F39" s="56" t="s">
+      <c r="F39" s="59" t="s">
         <v>224</v>
       </c>
       <c r="G39" s="5" t="s">
@@ -2987,30 +2987,30 @@
       <c r="H39" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I39" s="61"/>
-      <c r="J39" s="68"/>
+      <c r="I39" s="56"/>
+      <c r="J39" s="58"/>
     </row>
     <row r="40" spans="1:10" ht="15">
-      <c r="A40" s="47"/>
-      <c r="B40" s="47"/>
-      <c r="C40" s="47"/>
-      <c r="D40" s="61"/>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
+      <c r="A40" s="60"/>
+      <c r="B40" s="60"/>
+      <c r="C40" s="60"/>
+      <c r="D40" s="56"/>
+      <c r="E40" s="47"/>
+      <c r="F40" s="47"/>
       <c r="G40" s="5" t="s">
         <v>222</v>
       </c>
       <c r="H40" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="I40" s="61"/>
-      <c r="J40" s="68"/>
+      <c r="I40" s="56"/>
+      <c r="J40" s="58"/>
     </row>
     <row r="41" spans="1:10" ht="15">
-      <c r="A41" s="48"/>
-      <c r="B41" s="48"/>
-      <c r="C41" s="48"/>
-      <c r="D41" s="63"/>
+      <c r="A41" s="47"/>
+      <c r="B41" s="47"/>
+      <c r="C41" s="47"/>
+      <c r="D41" s="51"/>
       <c r="E41" s="32" t="s">
         <v>2</v>
       </c>
@@ -3023,26 +3023,26 @@
       <c r="H41" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="I41" s="61"/>
-      <c r="J41" s="68"/>
+      <c r="I41" s="56"/>
+      <c r="J41" s="58"/>
     </row>
     <row r="42" spans="1:10" ht="15">
-      <c r="A42" s="46">
+      <c r="A42" s="61">
         <v>12</v>
       </c>
-      <c r="B42" s="46" t="s">
+      <c r="B42" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C42" s="46" t="s">
+      <c r="C42" s="61" t="s">
         <v>270</v>
       </c>
-      <c r="D42" s="53" t="s">
+      <c r="D42" s="65" t="s">
         <v>272</v>
       </c>
-      <c r="E42" s="55" t="s">
+      <c r="E42" s="74" t="s">
         <v>182</v>
       </c>
-      <c r="F42" s="55" t="s">
+      <c r="F42" s="74" t="s">
         <v>180</v>
       </c>
       <c r="G42" s="6" t="s">
@@ -3051,68 +3051,68 @@
       <c r="H42" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="I42" s="61"/>
-      <c r="J42" s="68"/>
+      <c r="I42" s="56"/>
+      <c r="J42" s="58"/>
     </row>
     <row r="43" spans="1:10" ht="15">
-      <c r="A43" s="47"/>
-      <c r="B43" s="47"/>
-      <c r="C43" s="47"/>
-      <c r="D43" s="47"/>
-      <c r="E43" s="47"/>
-      <c r="F43" s="47"/>
+      <c r="A43" s="60"/>
+      <c r="B43" s="60"/>
+      <c r="C43" s="60"/>
+      <c r="D43" s="60"/>
+      <c r="E43" s="60"/>
+      <c r="F43" s="60"/>
       <c r="G43" s="6" t="s">
         <v>182</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="I43" s="61"/>
-      <c r="J43" s="68"/>
+      <c r="I43" s="56"/>
+      <c r="J43" s="58"/>
     </row>
     <row r="44" spans="1:10" ht="15">
-      <c r="A44" s="47"/>
-      <c r="B44" s="47"/>
-      <c r="C44" s="47"/>
-      <c r="D44" s="47"/>
-      <c r="E44" s="47"/>
-      <c r="F44" s="47"/>
+      <c r="A44" s="60"/>
+      <c r="B44" s="60"/>
+      <c r="C44" s="60"/>
+      <c r="D44" s="60"/>
+      <c r="E44" s="60"/>
+      <c r="F44" s="60"/>
       <c r="G44" s="6" t="s">
         <v>60</v>
       </c>
       <c r="H44" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="I44" s="61"/>
-      <c r="J44" s="68"/>
+      <c r="I44" s="56"/>
+      <c r="J44" s="58"/>
     </row>
     <row r="45" spans="1:10" ht="15">
-      <c r="A45" s="48"/>
-      <c r="B45" s="48"/>
-      <c r="C45" s="48"/>
-      <c r="D45" s="48"/>
-      <c r="E45" s="48"/>
-      <c r="F45" s="48"/>
+      <c r="A45" s="47"/>
+      <c r="B45" s="47"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="47"/>
+      <c r="E45" s="47"/>
+      <c r="F45" s="47"/>
       <c r="G45" s="6" t="s">
         <v>260</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="I45" s="61"/>
-      <c r="J45" s="68"/>
+      <c r="I45" s="56"/>
+      <c r="J45" s="58"/>
     </row>
     <row r="46" spans="1:10" ht="15">
-      <c r="A46" s="46">
+      <c r="A46" s="61">
         <v>13</v>
       </c>
-      <c r="B46" s="46" t="s">
+      <c r="B46" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C46" s="46" t="s">
+      <c r="C46" s="61" t="s">
         <v>273</v>
       </c>
-      <c r="D46" s="53" t="s">
+      <c r="D46" s="65" t="s">
         <v>274</v>
       </c>
       <c r="E46" s="11" t="s">
@@ -3127,18 +3127,18 @@
       <c r="H46" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="I46" s="61"/>
-      <c r="J46" s="68"/>
+      <c r="I46" s="56"/>
+      <c r="J46" s="58"/>
     </row>
     <row r="47" spans="1:10" ht="15">
-      <c r="A47" s="47"/>
-      <c r="B47" s="47"/>
-      <c r="C47" s="47"/>
-      <c r="D47" s="47"/>
-      <c r="E47" s="56" t="s">
+      <c r="A47" s="60"/>
+      <c r="B47" s="60"/>
+      <c r="C47" s="60"/>
+      <c r="D47" s="60"/>
+      <c r="E47" s="59" t="s">
         <v>78</v>
       </c>
-      <c r="F47" s="56" t="s">
+      <c r="F47" s="59" t="s">
         <v>79</v>
       </c>
       <c r="G47" s="5" t="s">
@@ -3147,58 +3147,58 @@
       <c r="H47" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="I47" s="61"/>
-      <c r="J47" s="68"/>
+      <c r="I47" s="56"/>
+      <c r="J47" s="58"/>
     </row>
     <row r="48" spans="1:10" ht="15">
-      <c r="A48" s="47"/>
-      <c r="B48" s="47"/>
-      <c r="C48" s="47"/>
-      <c r="D48" s="47"/>
-      <c r="E48" s="47"/>
-      <c r="F48" s="47"/>
+      <c r="A48" s="60"/>
+      <c r="B48" s="60"/>
+      <c r="C48" s="60"/>
+      <c r="D48" s="60"/>
+      <c r="E48" s="60"/>
+      <c r="F48" s="60"/>
       <c r="G48" s="6" t="s">
         <v>214</v>
       </c>
       <c r="H48" s="34" t="s">
         <v>215</v>
       </c>
-      <c r="I48" s="61"/>
-      <c r="J48" s="68"/>
+      <c r="I48" s="56"/>
+      <c r="J48" s="58"/>
     </row>
     <row r="49" spans="1:10" ht="15">
-      <c r="A49" s="48"/>
-      <c r="B49" s="48"/>
-      <c r="C49" s="48"/>
-      <c r="D49" s="48"/>
-      <c r="E49" s="47"/>
-      <c r="F49" s="47"/>
+      <c r="A49" s="47"/>
+      <c r="B49" s="47"/>
+      <c r="C49" s="47"/>
+      <c r="D49" s="47"/>
+      <c r="E49" s="60"/>
+      <c r="F49" s="60"/>
       <c r="G49" s="6" t="s">
         <v>218</v>
       </c>
       <c r="H49" s="34" t="s">
         <v>219</v>
       </c>
-      <c r="I49" s="61"/>
-      <c r="J49" s="68"/>
+      <c r="I49" s="56"/>
+      <c r="J49" s="58"/>
     </row>
     <row r="50" spans="1:10" ht="15">
-      <c r="A50" s="46">
+      <c r="A50" s="61">
         <v>14</v>
       </c>
-      <c r="B50" s="46" t="s">
+      <c r="B50" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C50" s="46" t="s">
+      <c r="C50" s="61" t="s">
         <v>275</v>
       </c>
-      <c r="D50" s="53" t="s">
+      <c r="D50" s="65" t="s">
         <v>276</v>
       </c>
-      <c r="E50" s="51" t="s">
+      <c r="E50" s="46" t="s">
         <v>184</v>
       </c>
-      <c r="F50" s="51" t="s">
+      <c r="F50" s="46" t="s">
         <v>185</v>
       </c>
       <c r="G50" s="6" t="s">
@@ -3207,58 +3207,58 @@
       <c r="H50" s="34" t="s">
         <v>185</v>
       </c>
-      <c r="I50" s="61"/>
-      <c r="J50" s="68"/>
+      <c r="I50" s="56"/>
+      <c r="J50" s="58"/>
     </row>
     <row r="51" spans="1:10" ht="15">
-      <c r="A51" s="47"/>
-      <c r="B51" s="47"/>
-      <c r="C51" s="47"/>
-      <c r="D51" s="47"/>
-      <c r="E51" s="47"/>
-      <c r="F51" s="47"/>
+      <c r="A51" s="60"/>
+      <c r="B51" s="60"/>
+      <c r="C51" s="60"/>
+      <c r="D51" s="60"/>
+      <c r="E51" s="60"/>
+      <c r="F51" s="60"/>
       <c r="G51" s="6" t="s">
         <v>43</v>
       </c>
       <c r="H51" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="I51" s="61"/>
-      <c r="J51" s="68"/>
+      <c r="I51" s="56"/>
+      <c r="J51" s="58"/>
     </row>
     <row r="52" spans="1:10" ht="15">
-      <c r="A52" s="48"/>
-      <c r="B52" s="48"/>
-      <c r="C52" s="48"/>
-      <c r="D52" s="48"/>
-      <c r="E52" s="47"/>
-      <c r="F52" s="47"/>
+      <c r="A52" s="47"/>
+      <c r="B52" s="47"/>
+      <c r="C52" s="47"/>
+      <c r="D52" s="47"/>
+      <c r="E52" s="60"/>
+      <c r="F52" s="60"/>
       <c r="G52" s="6" t="s">
         <v>139</v>
       </c>
       <c r="H52" s="34" t="s">
         <v>140</v>
       </c>
-      <c r="I52" s="61"/>
-      <c r="J52" s="68"/>
+      <c r="I52" s="56"/>
+      <c r="J52" s="58"/>
     </row>
     <row r="53" spans="1:10" ht="35.25" customHeight="1">
-      <c r="A53" s="46">
+      <c r="A53" s="61">
         <v>15</v>
       </c>
-      <c r="B53" s="49" t="s">
+      <c r="B53" s="62" t="s">
         <v>98</v>
       </c>
-      <c r="C53" s="49" t="s">
+      <c r="C53" s="62" t="s">
         <v>277</v>
       </c>
-      <c r="D53" s="50" t="s">
+      <c r="D53" s="63" t="s">
         <v>278</v>
       </c>
-      <c r="E53" s="51" t="s">
+      <c r="E53" s="46" t="s">
         <v>76</v>
       </c>
-      <c r="F53" s="51" t="s">
+      <c r="F53" s="46" t="s">
         <v>94</v>
       </c>
       <c r="G53" s="5" t="s">
@@ -3267,24 +3267,24 @@
       <c r="H53" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="I53" s="61"/>
-      <c r="J53" s="68"/>
+      <c r="I53" s="56"/>
+      <c r="J53" s="58"/>
     </row>
     <row r="54" spans="1:10" ht="28.5" customHeight="1">
-      <c r="A54" s="48"/>
-      <c r="B54" s="48"/>
-      <c r="C54" s="48"/>
-      <c r="D54" s="48"/>
-      <c r="E54" s="48"/>
-      <c r="F54" s="48"/>
+      <c r="A54" s="47"/>
+      <c r="B54" s="47"/>
+      <c r="C54" s="47"/>
+      <c r="D54" s="47"/>
+      <c r="E54" s="47"/>
+      <c r="F54" s="47"/>
       <c r="G54" s="5" t="s">
         <v>188</v>
       </c>
       <c r="H54" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="I54" s="61"/>
-      <c r="J54" s="68"/>
+      <c r="I54" s="56"/>
+      <c r="J54" s="58"/>
     </row>
     <row r="55" spans="1:10" ht="30">
       <c r="A55" s="8">
@@ -3311,18 +3311,18 @@
       <c r="H55" s="34" t="s">
         <v>205</v>
       </c>
-      <c r="I55" s="63"/>
-      <c r="J55" s="69"/>
+      <c r="I55" s="51"/>
+      <c r="J55" s="53"/>
     </row>
     <row r="56" spans="1:10" ht="15">
-      <c r="A56" s="46"/>
-      <c r="B56" s="46" t="s">
+      <c r="A56" s="61"/>
+      <c r="B56" s="61" t="s">
         <v>55</v>
       </c>
-      <c r="C56" s="46" t="s">
+      <c r="C56" s="61" t="s">
         <v>281</v>
       </c>
-      <c r="D56" s="53" t="s">
+      <c r="D56" s="65" t="s">
         <v>282</v>
       </c>
       <c r="E56" s="11" t="s">
@@ -3331,28 +3331,28 @@
       <c r="F56" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="G56" s="66" t="s">
+      <c r="G56" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="H56" s="70"/>
-      <c r="I56" s="70"/>
-      <c r="J56" s="67"/>
+      <c r="H56" s="49"/>
+      <c r="I56" s="49"/>
+      <c r="J56" s="50"/>
     </row>
     <row r="57" spans="1:10" ht="24.75" customHeight="1">
-      <c r="A57" s="48"/>
-      <c r="B57" s="48"/>
-      <c r="C57" s="48"/>
-      <c r="D57" s="48"/>
+      <c r="A57" s="47"/>
+      <c r="B57" s="47"/>
+      <c r="C57" s="47"/>
+      <c r="D57" s="47"/>
       <c r="E57" s="5" t="s">
         <v>72</v>
       </c>
       <c r="F57" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G57" s="63"/>
-      <c r="H57" s="71"/>
-      <c r="I57" s="71"/>
-      <c r="J57" s="69"/>
+      <c r="G57" s="51"/>
+      <c r="H57" s="52"/>
+      <c r="I57" s="52"/>
+      <c r="J57" s="53"/>
     </row>
     <row r="58" spans="1:10" ht="30">
       <c r="A58" s="8">
@@ -3367,18 +3367,18 @@
       <c r="D58" s="35" t="s">
         <v>284</v>
       </c>
-      <c r="E58" s="51" t="s">
+      <c r="E58" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="F58" s="51" t="s">
+      <c r="F58" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="G58" s="72" t="s">
+      <c r="G58" s="54" t="s">
         <v>30</v>
       </c>
-      <c r="H58" s="73"/>
-      <c r="I58" s="73"/>
-      <c r="J58" s="65"/>
+      <c r="H58" s="68"/>
+      <c r="I58" s="68"/>
+      <c r="J58" s="55"/>
     </row>
     <row r="59" spans="1:10" ht="45">
       <c r="A59" s="8">
@@ -3393,24 +3393,24 @@
       <c r="D59" s="36" t="s">
         <v>287</v>
       </c>
-      <c r="E59" s="48"/>
-      <c r="F59" s="48"/>
-      <c r="G59" s="74"/>
-      <c r="H59" s="73"/>
-      <c r="I59" s="73"/>
-      <c r="J59" s="65"/>
+      <c r="E59" s="47"/>
+      <c r="F59" s="47"/>
+      <c r="G59" s="69"/>
+      <c r="H59" s="68"/>
+      <c r="I59" s="68"/>
+      <c r="J59" s="55"/>
     </row>
     <row r="60" spans="1:10" ht="15">
-      <c r="A60" s="46">
+      <c r="A60" s="61">
         <v>17</v>
       </c>
-      <c r="B60" s="49" t="s">
+      <c r="B60" s="62" t="s">
         <v>285</v>
       </c>
-      <c r="C60" s="49" t="s">
+      <c r="C60" s="62" t="s">
         <v>288</v>
       </c>
-      <c r="D60" s="50" t="s">
+      <c r="D60" s="63" t="s">
         <v>289</v>
       </c>
       <c r="E60" s="11" t="s">
@@ -3425,14 +3425,14 @@
       <c r="H60" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="I60" s="75"/>
-      <c r="J60" s="67"/>
+      <c r="I60" s="70"/>
+      <c r="J60" s="50"/>
     </row>
     <row r="61" spans="1:10" ht="25.5" customHeight="1">
-      <c r="A61" s="47"/>
-      <c r="B61" s="47"/>
-      <c r="C61" s="47"/>
-      <c r="D61" s="47"/>
+      <c r="A61" s="60"/>
+      <c r="B61" s="60"/>
+      <c r="C61" s="60"/>
+      <c r="D61" s="60"/>
       <c r="E61" s="11" t="s">
         <v>114</v>
       </c>
@@ -3445,14 +3445,14 @@
       <c r="H61" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="I61" s="61"/>
-      <c r="J61" s="68"/>
+      <c r="I61" s="56"/>
+      <c r="J61" s="58"/>
     </row>
     <row r="62" spans="1:10" ht="25.5" customHeight="1">
-      <c r="A62" s="48"/>
-      <c r="B62" s="48"/>
-      <c r="C62" s="48"/>
-      <c r="D62" s="48"/>
+      <c r="A62" s="47"/>
+      <c r="B62" s="47"/>
+      <c r="C62" s="47"/>
+      <c r="D62" s="47"/>
       <c r="E62" s="11" t="s">
         <v>254</v>
       </c>
@@ -3465,30 +3465,30 @@
       <c r="H62" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="I62" s="63"/>
-      <c r="J62" s="69"/>
+      <c r="I62" s="51"/>
+      <c r="J62" s="53"/>
     </row>
     <row r="63" spans="1:10" ht="15">
-      <c r="A63" s="46">
+      <c r="A63" s="61">
         <v>19</v>
       </c>
-      <c r="B63" s="46" t="s">
+      <c r="B63" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C63" s="46" t="s">
+      <c r="C63" s="61" t="s">
         <v>290</v>
       </c>
-      <c r="D63" s="52" t="s">
+      <c r="D63" s="64" t="s">
         <v>291</v>
       </c>
-      <c r="E63" s="56" t="s">
+      <c r="E63" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="F63" s="56" t="s">
+      <c r="F63" s="59" t="s">
         <v>195</v>
       </c>
-      <c r="G63" s="66"/>
-      <c r="H63" s="67"/>
+      <c r="G63" s="48"/>
+      <c r="H63" s="50"/>
       <c r="I63" s="5" t="s">
         <v>99</v>
       </c>
@@ -3497,14 +3497,14 @@
       </c>
     </row>
     <row r="64" spans="1:10" ht="15">
-      <c r="A64" s="48"/>
-      <c r="B64" s="48"/>
-      <c r="C64" s="48"/>
-      <c r="D64" s="48"/>
-      <c r="E64" s="48"/>
-      <c r="F64" s="48"/>
-      <c r="G64" s="63"/>
-      <c r="H64" s="69"/>
+      <c r="A64" s="47"/>
+      <c r="B64" s="47"/>
+      <c r="C64" s="47"/>
+      <c r="D64" s="47"/>
+      <c r="E64" s="47"/>
+      <c r="F64" s="47"/>
+      <c r="G64" s="51"/>
+      <c r="H64" s="53"/>
       <c r="I64" s="5" t="s">
         <v>40</v>
       </c>
@@ -3513,14 +3513,14 @@
       </c>
     </row>
     <row r="65" spans="1:10" ht="15">
-      <c r="A65" s="46"/>
-      <c r="B65" s="46" t="s">
+      <c r="A65" s="61"/>
+      <c r="B65" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C65" s="46" t="s">
+      <c r="C65" s="61" t="s">
         <v>292</v>
       </c>
-      <c r="D65" s="52" t="s">
+      <c r="D65" s="64" t="s">
         <v>293</v>
       </c>
       <c r="E65" s="16" t="s">
@@ -3543,10 +3543,10 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="15">
-      <c r="A66" s="48"/>
-      <c r="B66" s="48"/>
-      <c r="C66" s="48"/>
-      <c r="D66" s="48"/>
+      <c r="A66" s="47"/>
+      <c r="B66" s="47"/>
+      <c r="C66" s="47"/>
+      <c r="D66" s="47"/>
       <c r="E66" s="5" t="s">
         <v>196</v>
       </c>
@@ -3567,16 +3567,16 @@
       </c>
     </row>
     <row r="67" spans="1:10" ht="15">
-      <c r="A67" s="46">
+      <c r="A67" s="61">
         <v>21</v>
       </c>
-      <c r="B67" s="46" t="s">
+      <c r="B67" s="61" t="s">
         <v>294</v>
       </c>
-      <c r="C67" s="46" t="s">
+      <c r="C67" s="61" t="s">
         <v>295</v>
       </c>
-      <c r="D67" s="52" t="s">
+      <c r="D67" s="64" t="s">
         <v>296</v>
       </c>
       <c r="E67" s="11" t="s">
@@ -3585,38 +3585,38 @@
       <c r="F67" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="G67" s="66"/>
-      <c r="H67" s="67"/>
-      <c r="I67" s="66" t="s">
+      <c r="G67" s="48"/>
+      <c r="H67" s="50"/>
+      <c r="I67" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="J67" s="67"/>
+      <c r="J67" s="50"/>
     </row>
     <row r="68" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A68" s="48"/>
-      <c r="B68" s="47"/>
-      <c r="C68" s="48"/>
-      <c r="D68" s="48"/>
+      <c r="A68" s="47"/>
+      <c r="B68" s="60"/>
+      <c r="C68" s="47"/>
+      <c r="D68" s="47"/>
       <c r="E68" s="5" t="s">
         <v>116</v>
       </c>
       <c r="F68" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="G68" s="61"/>
-      <c r="H68" s="68"/>
-      <c r="I68" s="61"/>
-      <c r="J68" s="68"/>
+      <c r="G68" s="56"/>
+      <c r="H68" s="58"/>
+      <c r="I68" s="56"/>
+      <c r="J68" s="58"/>
     </row>
     <row r="69" spans="1:10" ht="15">
       <c r="A69" s="8">
         <v>22</v>
       </c>
-      <c r="B69" s="47"/>
-      <c r="C69" s="46" t="s">
+      <c r="B69" s="60"/>
+      <c r="C69" s="61" t="s">
         <v>297</v>
       </c>
-      <c r="D69" s="52" t="s">
+      <c r="D69" s="64" t="s">
         <v>298</v>
       </c>
       <c r="E69" s="11" t="s">
@@ -3625,38 +3625,38 @@
       <c r="F69" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="G69" s="61"/>
-      <c r="H69" s="68"/>
-      <c r="I69" s="61"/>
-      <c r="J69" s="68"/>
+      <c r="G69" s="56"/>
+      <c r="H69" s="58"/>
+      <c r="I69" s="56"/>
+      <c r="J69" s="58"/>
     </row>
     <row r="70" spans="1:10" ht="30">
       <c r="A70" s="8"/>
-      <c r="B70" s="48"/>
-      <c r="C70" s="48"/>
-      <c r="D70" s="48"/>
+      <c r="B70" s="47"/>
+      <c r="C70" s="47"/>
+      <c r="D70" s="47"/>
       <c r="E70" s="5" t="s">
         <v>116</v>
       </c>
       <c r="F70" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="G70" s="61"/>
-      <c r="H70" s="68"/>
-      <c r="I70" s="61"/>
-      <c r="J70" s="68"/>
+      <c r="G70" s="56"/>
+      <c r="H70" s="58"/>
+      <c r="I70" s="56"/>
+      <c r="J70" s="58"/>
     </row>
     <row r="71" spans="1:10" ht="15">
-      <c r="A71" s="46">
+      <c r="A71" s="61">
         <v>23</v>
       </c>
-      <c r="B71" s="46" t="s">
+      <c r="B71" s="61" t="s">
         <v>299</v>
       </c>
-      <c r="C71" s="46" t="s">
+      <c r="C71" s="61" t="s">
         <v>300</v>
       </c>
-      <c r="D71" s="52" t="s">
+      <c r="D71" s="64" t="s">
         <v>301</v>
       </c>
       <c r="E71" s="11" t="s">
@@ -3665,36 +3665,36 @@
       <c r="F71" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="G71" s="61"/>
-      <c r="H71" s="68"/>
-      <c r="I71" s="61"/>
-      <c r="J71" s="68"/>
+      <c r="G71" s="56"/>
+      <c r="H71" s="58"/>
+      <c r="I71" s="56"/>
+      <c r="J71" s="58"/>
     </row>
     <row r="72" spans="1:10" ht="30">
-      <c r="A72" s="48"/>
-      <c r="B72" s="47"/>
-      <c r="C72" s="48"/>
-      <c r="D72" s="48"/>
+      <c r="A72" s="47"/>
+      <c r="B72" s="60"/>
+      <c r="C72" s="47"/>
+      <c r="D72" s="47"/>
       <c r="E72" s="5" t="s">
         <v>116</v>
       </c>
       <c r="F72" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="G72" s="61"/>
-      <c r="H72" s="68"/>
-      <c r="I72" s="61"/>
-      <c r="J72" s="68"/>
+      <c r="G72" s="56"/>
+      <c r="H72" s="58"/>
+      <c r="I72" s="56"/>
+      <c r="J72" s="58"/>
     </row>
     <row r="73" spans="1:10" ht="15">
-      <c r="A73" s="46">
+      <c r="A73" s="61">
         <v>24</v>
       </c>
-      <c r="B73" s="47"/>
-      <c r="C73" s="46" t="s">
+      <c r="B73" s="60"/>
+      <c r="C73" s="61" t="s">
         <v>302</v>
       </c>
-      <c r="D73" s="52" t="s">
+      <c r="D73" s="64" t="s">
         <v>303</v>
       </c>
       <c r="E73" s="11" t="s">
@@ -3703,26 +3703,26 @@
       <c r="F73" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="G73" s="61"/>
-      <c r="H73" s="68"/>
-      <c r="I73" s="61"/>
-      <c r="J73" s="68"/>
+      <c r="G73" s="56"/>
+      <c r="H73" s="58"/>
+      <c r="I73" s="56"/>
+      <c r="J73" s="58"/>
     </row>
     <row r="74" spans="1:10" ht="30">
-      <c r="A74" s="48"/>
-      <c r="B74" s="48"/>
-      <c r="C74" s="48"/>
-      <c r="D74" s="48"/>
+      <c r="A74" s="47"/>
+      <c r="B74" s="47"/>
+      <c r="C74" s="47"/>
+      <c r="D74" s="47"/>
       <c r="E74" s="5" t="s">
         <v>116</v>
       </c>
       <c r="F74" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="G74" s="63"/>
-      <c r="H74" s="69"/>
-      <c r="I74" s="61"/>
-      <c r="J74" s="68"/>
+      <c r="G74" s="51"/>
+      <c r="H74" s="53"/>
+      <c r="I74" s="56"/>
+      <c r="J74" s="58"/>
     </row>
     <row r="75" spans="1:10" ht="15">
       <c r="A75" s="8">
@@ -3743,30 +3743,30 @@
       <c r="F75" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="G75" s="72" t="s">
+      <c r="G75" s="54" t="s">
         <v>30</v>
       </c>
-      <c r="H75" s="65"/>
-      <c r="I75" s="61"/>
-      <c r="J75" s="68"/>
+      <c r="H75" s="55"/>
+      <c r="I75" s="56"/>
+      <c r="J75" s="58"/>
     </row>
     <row r="76" spans="1:10" ht="42" customHeight="1">
-      <c r="A76" s="46">
+      <c r="A76" s="61">
         <v>25</v>
       </c>
-      <c r="B76" s="46" t="s">
+      <c r="B76" s="61" t="s">
         <v>306</v>
       </c>
-      <c r="C76" s="46" t="s">
+      <c r="C76" s="61" t="s">
         <v>307</v>
       </c>
-      <c r="D76" s="53" t="s">
+      <c r="D76" s="65" t="s">
         <v>276</v>
       </c>
-      <c r="E76" s="51" t="s">
+      <c r="E76" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="F76" s="51" t="s">
+      <c r="F76" s="46" t="s">
         <v>27</v>
       </c>
       <c r="G76" s="5" t="s">
@@ -3775,36 +3775,36 @@
       <c r="H76" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I76" s="61"/>
-      <c r="J76" s="68"/>
+      <c r="I76" s="56"/>
+      <c r="J76" s="58"/>
     </row>
     <row r="77" spans="1:10" ht="15">
-      <c r="A77" s="48"/>
-      <c r="B77" s="48"/>
-      <c r="C77" s="48"/>
-      <c r="D77" s="48"/>
-      <c r="E77" s="48"/>
-      <c r="F77" s="48"/>
+      <c r="A77" s="47"/>
+      <c r="B77" s="47"/>
+      <c r="C77" s="47"/>
+      <c r="D77" s="47"/>
+      <c r="E77" s="47"/>
+      <c r="F77" s="47"/>
       <c r="G77" s="5" t="s">
         <v>139</v>
       </c>
       <c r="H77" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="I77" s="61"/>
-      <c r="J77" s="68"/>
+      <c r="I77" s="56"/>
+      <c r="J77" s="58"/>
     </row>
     <row r="78" spans="1:10" ht="30">
-      <c r="A78" s="46">
+      <c r="A78" s="61">
         <v>27</v>
       </c>
-      <c r="B78" s="46" t="s">
+      <c r="B78" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="C78" s="46" t="s">
+      <c r="C78" s="61" t="s">
         <v>308</v>
       </c>
-      <c r="D78" s="53" t="s">
+      <c r="D78" s="65" t="s">
         <v>309</v>
       </c>
       <c r="E78" s="5" t="s">
@@ -3819,18 +3819,18 @@
       <c r="H78" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="I78" s="61"/>
-      <c r="J78" s="68"/>
+      <c r="I78" s="56"/>
+      <c r="J78" s="58"/>
     </row>
     <row r="79" spans="1:10" ht="15">
-      <c r="A79" s="47"/>
-      <c r="B79" s="47"/>
-      <c r="C79" s="47"/>
-      <c r="D79" s="47"/>
-      <c r="E79" s="56" t="s">
+      <c r="A79" s="60"/>
+      <c r="B79" s="60"/>
+      <c r="C79" s="60"/>
+      <c r="D79" s="60"/>
+      <c r="E79" s="59" t="s">
         <v>256</v>
       </c>
-      <c r="F79" s="56" t="s">
+      <c r="F79" s="59" t="s">
         <v>257</v>
       </c>
       <c r="G79" s="5" t="s">
@@ -3839,84 +3839,84 @@
       <c r="H79" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="I79" s="61"/>
-      <c r="J79" s="68"/>
+      <c r="I79" s="56"/>
+      <c r="J79" s="58"/>
     </row>
     <row r="80" spans="1:10" ht="15">
-      <c r="A80" s="47"/>
-      <c r="B80" s="47"/>
-      <c r="C80" s="47"/>
-      <c r="D80" s="47"/>
-      <c r="E80" s="47"/>
-      <c r="F80" s="47"/>
+      <c r="A80" s="60"/>
+      <c r="B80" s="60"/>
+      <c r="C80" s="60"/>
+      <c r="D80" s="60"/>
+      <c r="E80" s="60"/>
+      <c r="F80" s="60"/>
       <c r="G80" s="5" t="s">
         <v>247</v>
       </c>
       <c r="H80" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="I80" s="61"/>
-      <c r="J80" s="68"/>
+      <c r="I80" s="56"/>
+      <c r="J80" s="58"/>
     </row>
     <row r="81" spans="1:10" ht="15">
-      <c r="A81" s="48"/>
-      <c r="B81" s="48"/>
-      <c r="C81" s="48"/>
-      <c r="D81" s="48"/>
-      <c r="E81" s="48"/>
-      <c r="F81" s="48"/>
+      <c r="A81" s="47"/>
+      <c r="B81" s="47"/>
+      <c r="C81" s="47"/>
+      <c r="D81" s="47"/>
+      <c r="E81" s="47"/>
+      <c r="F81" s="47"/>
       <c r="G81" s="5" t="s">
         <v>237</v>
       </c>
       <c r="H81" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="I81" s="63"/>
-      <c r="J81" s="69"/>
+      <c r="I81" s="51"/>
+      <c r="J81" s="53"/>
     </row>
     <row r="82" spans="1:10" ht="13">
-      <c r="A82" s="46">
+      <c r="A82" s="61">
         <v>28</v>
       </c>
-      <c r="B82" s="49" t="s">
+      <c r="B82" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="C82" s="49" t="s">
+      <c r="C82" s="62" t="s">
         <v>310</v>
       </c>
-      <c r="D82" s="50" t="s">
+      <c r="D82" s="63" t="s">
         <v>311</v>
       </c>
-      <c r="E82" s="51" t="s">
+      <c r="E82" s="46" t="s">
         <v>228</v>
       </c>
-      <c r="F82" s="51" t="s">
+      <c r="F82" s="46" t="s">
         <v>231</v>
       </c>
-      <c r="G82" s="66" t="s">
+      <c r="G82" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="H82" s="70"/>
-      <c r="I82" s="70"/>
-      <c r="J82" s="67"/>
+      <c r="H82" s="49"/>
+      <c r="I82" s="49"/>
+      <c r="J82" s="50"/>
     </row>
     <row r="83" spans="1:10" ht="13">
-      <c r="A83" s="48"/>
-      <c r="B83" s="48"/>
-      <c r="C83" s="48"/>
-      <c r="D83" s="48"/>
-      <c r="E83" s="48"/>
-      <c r="F83" s="48"/>
-      <c r="G83" s="63"/>
-      <c r="H83" s="71"/>
-      <c r="I83" s="71"/>
-      <c r="J83" s="69"/>
+      <c r="A83" s="47"/>
+      <c r="B83" s="47"/>
+      <c r="C83" s="47"/>
+      <c r="D83" s="47"/>
+      <c r="E83" s="47"/>
+      <c r="F83" s="47"/>
+      <c r="G83" s="51"/>
+      <c r="H83" s="52"/>
+      <c r="I83" s="52"/>
+      <c r="J83" s="53"/>
     </row>
     <row r="84" spans="1:10" ht="30">
       <c r="A84" s="8">
         <v>29</v>
       </c>
-      <c r="B84" s="46" t="s">
+      <c r="B84" s="61" t="s">
         <v>312</v>
       </c>
       <c r="C84" s="8" t="s">
@@ -3931,18 +3931,18 @@
       <c r="F84" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="G84" s="66" t="s">
+      <c r="G84" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="H84" s="70"/>
-      <c r="I84" s="70"/>
-      <c r="J84" s="67"/>
+      <c r="H84" s="49"/>
+      <c r="I84" s="49"/>
+      <c r="J84" s="50"/>
     </row>
     <row r="85" spans="1:10" ht="15">
       <c r="A85" s="8">
         <v>30</v>
       </c>
-      <c r="B85" s="48"/>
+      <c r="B85" s="47"/>
       <c r="C85" s="8" t="s">
         <v>315</v>
       </c>
@@ -3955,10 +3955,10 @@
       <c r="F85" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G85" s="63"/>
-      <c r="H85" s="71"/>
-      <c r="I85" s="71"/>
-      <c r="J85" s="69"/>
+      <c r="G85" s="51"/>
+      <c r="H85" s="52"/>
+      <c r="I85" s="52"/>
+      <c r="J85" s="53"/>
     </row>
     <row r="86" spans="1:10" ht="45">
       <c r="A86" s="8">
@@ -3985,16 +3985,16 @@
       <c r="H86" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="I86" s="72" t="s">
+      <c r="I86" s="54" t="s">
         <v>30</v>
       </c>
-      <c r="J86" s="65"/>
+      <c r="J86" s="55"/>
     </row>
     <row r="87" spans="1:10" ht="15">
       <c r="A87" s="8">
         <v>32</v>
       </c>
-      <c r="B87" s="46" t="s">
+      <c r="B87" s="61" t="s">
         <v>312</v>
       </c>
       <c r="C87" s="8" t="s">
@@ -4003,72 +4003,72 @@
       <c r="D87" s="35" t="s">
         <v>321</v>
       </c>
-      <c r="E87" s="51" t="s">
+      <c r="E87" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="F87" s="51" t="s">
+      <c r="F87" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="G87" s="66" t="s">
+      <c r="G87" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="H87" s="70"/>
-      <c r="I87" s="70"/>
-      <c r="J87" s="67"/>
+      <c r="H87" s="49"/>
+      <c r="I87" s="49"/>
+      <c r="J87" s="50"/>
     </row>
     <row r="88" spans="1:10" ht="15">
       <c r="A88" s="8">
         <v>33</v>
       </c>
-      <c r="B88" s="47"/>
+      <c r="B88" s="60"/>
       <c r="C88" s="8" t="s">
         <v>322</v>
       </c>
       <c r="D88" s="35" t="s">
         <v>323</v>
       </c>
-      <c r="E88" s="47"/>
-      <c r="F88" s="47"/>
-      <c r="G88" s="61"/>
-      <c r="H88" s="79"/>
-      <c r="I88" s="79"/>
-      <c r="J88" s="68"/>
+      <c r="E88" s="60"/>
+      <c r="F88" s="60"/>
+      <c r="G88" s="56"/>
+      <c r="H88" s="57"/>
+      <c r="I88" s="57"/>
+      <c r="J88" s="58"/>
     </row>
     <row r="89" spans="1:10" ht="15">
       <c r="A89" s="8">
         <v>34</v>
       </c>
-      <c r="B89" s="47"/>
+      <c r="B89" s="60"/>
       <c r="C89" s="8" t="s">
         <v>324</v>
       </c>
       <c r="D89" s="35" t="s">
         <v>325</v>
       </c>
-      <c r="E89" s="47"/>
-      <c r="F89" s="47"/>
-      <c r="G89" s="61"/>
-      <c r="H89" s="79"/>
-      <c r="I89" s="79"/>
-      <c r="J89" s="68"/>
+      <c r="E89" s="60"/>
+      <c r="F89" s="60"/>
+      <c r="G89" s="56"/>
+      <c r="H89" s="57"/>
+      <c r="I89" s="57"/>
+      <c r="J89" s="58"/>
     </row>
     <row r="90" spans="1:10" ht="15">
       <c r="A90" s="8">
         <v>35</v>
       </c>
-      <c r="B90" s="48"/>
+      <c r="B90" s="47"/>
       <c r="C90" s="8" t="s">
         <v>326</v>
       </c>
       <c r="D90" s="35" t="s">
         <v>327</v>
       </c>
-      <c r="E90" s="48"/>
-      <c r="F90" s="48"/>
-      <c r="G90" s="61"/>
-      <c r="H90" s="79"/>
-      <c r="I90" s="79"/>
-      <c r="J90" s="68"/>
+      <c r="E90" s="47"/>
+      <c r="F90" s="47"/>
+      <c r="G90" s="56"/>
+      <c r="H90" s="57"/>
+      <c r="I90" s="57"/>
+      <c r="J90" s="58"/>
     </row>
     <row r="91" spans="1:10" ht="30">
       <c r="A91" s="8">
@@ -4089,10 +4089,10 @@
       <c r="F91" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="G91" s="61"/>
-      <c r="H91" s="79"/>
-      <c r="I91" s="79"/>
-      <c r="J91" s="68"/>
+      <c r="G91" s="56"/>
+      <c r="H91" s="57"/>
+      <c r="I91" s="57"/>
+      <c r="J91" s="58"/>
     </row>
     <row r="92" spans="1:10" ht="30">
       <c r="A92" s="8">
@@ -4113,16 +4113,16 @@
       <c r="F92" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="G92" s="63"/>
-      <c r="H92" s="71"/>
-      <c r="I92" s="71"/>
-      <c r="J92" s="69"/>
+      <c r="G92" s="51"/>
+      <c r="H92" s="52"/>
+      <c r="I92" s="52"/>
+      <c r="J92" s="53"/>
     </row>
     <row r="93" spans="1:10" ht="18.75" customHeight="1">
       <c r="A93" s="8">
         <v>38</v>
       </c>
-      <c r="B93" s="57" t="s">
+      <c r="B93" s="66" t="s">
         <v>332</v>
       </c>
       <c r="C93" s="8" t="s">
@@ -4143,16 +4143,16 @@
       <c r="H93" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="I93" s="66" t="s">
+      <c r="I93" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="J93" s="67"/>
+      <c r="J93" s="50"/>
     </row>
     <row r="94" spans="1:10" ht="18.75" customHeight="1">
       <c r="A94" s="8">
         <v>39</v>
       </c>
-      <c r="B94" s="47"/>
+      <c r="B94" s="60"/>
       <c r="C94" s="8" t="s">
         <v>335</v>
       </c>
@@ -4171,14 +4171,14 @@
       <c r="H94" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="I94" s="61"/>
-      <c r="J94" s="68"/>
+      <c r="I94" s="56"/>
+      <c r="J94" s="58"/>
     </row>
     <row r="95" spans="1:10" ht="18.75" customHeight="1">
       <c r="A95" s="8">
         <v>40</v>
       </c>
-      <c r="B95" s="47"/>
+      <c r="B95" s="60"/>
       <c r="C95" s="8" t="s">
         <v>337</v>
       </c>
@@ -4197,18 +4197,18 @@
       <c r="H95" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="I95" s="61"/>
-      <c r="J95" s="68"/>
+      <c r="I95" s="56"/>
+      <c r="J95" s="58"/>
     </row>
     <row r="96" spans="1:10" ht="15">
-      <c r="A96" s="46">
+      <c r="A96" s="61">
         <v>41</v>
       </c>
-      <c r="B96" s="47"/>
-      <c r="C96" s="46" t="s">
+      <c r="B96" s="60"/>
+      <c r="C96" s="61" t="s">
         <v>339</v>
       </c>
-      <c r="D96" s="53" t="s">
+      <c r="D96" s="65" t="s">
         <v>340</v>
       </c>
       <c r="E96" s="5" t="s">
@@ -4217,80 +4217,80 @@
       <c r="F96" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G96" s="66"/>
-      <c r="H96" s="67"/>
-      <c r="I96" s="61"/>
-      <c r="J96" s="68"/>
+      <c r="G96" s="48"/>
+      <c r="H96" s="50"/>
+      <c r="I96" s="56"/>
+      <c r="J96" s="58"/>
     </row>
     <row r="97" spans="1:10" ht="15">
-      <c r="A97" s="47"/>
-      <c r="B97" s="47"/>
-      <c r="C97" s="47"/>
-      <c r="D97" s="47"/>
+      <c r="A97" s="60"/>
+      <c r="B97" s="60"/>
+      <c r="C97" s="60"/>
+      <c r="D97" s="60"/>
       <c r="E97" s="5" t="s">
         <v>110</v>
       </c>
       <c r="F97" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="G97" s="61"/>
-      <c r="H97" s="68"/>
-      <c r="I97" s="61"/>
-      <c r="J97" s="68"/>
+      <c r="G97" s="56"/>
+      <c r="H97" s="58"/>
+      <c r="I97" s="56"/>
+      <c r="J97" s="58"/>
     </row>
     <row r="98" spans="1:10" ht="15">
-      <c r="A98" s="47"/>
-      <c r="B98" s="47"/>
-      <c r="C98" s="47"/>
-      <c r="D98" s="47"/>
+      <c r="A98" s="60"/>
+      <c r="B98" s="60"/>
+      <c r="C98" s="60"/>
+      <c r="D98" s="60"/>
       <c r="E98" s="5" t="s">
         <v>262</v>
       </c>
       <c r="F98" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="G98" s="61"/>
-      <c r="H98" s="68"/>
-      <c r="I98" s="61"/>
-      <c r="J98" s="68"/>
+      <c r="G98" s="56"/>
+      <c r="H98" s="58"/>
+      <c r="I98" s="56"/>
+      <c r="J98" s="58"/>
     </row>
     <row r="99" spans="1:10" ht="15">
-      <c r="A99" s="47"/>
-      <c r="B99" s="47"/>
-      <c r="C99" s="47"/>
-      <c r="D99" s="47"/>
+      <c r="A99" s="60"/>
+      <c r="B99" s="60"/>
+      <c r="C99" s="60"/>
+      <c r="D99" s="60"/>
       <c r="E99" s="5" t="s">
         <v>264</v>
       </c>
       <c r="F99" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="G99" s="61"/>
-      <c r="H99" s="68"/>
-      <c r="I99" s="61"/>
-      <c r="J99" s="68"/>
+      <c r="G99" s="56"/>
+      <c r="H99" s="58"/>
+      <c r="I99" s="56"/>
+      <c r="J99" s="58"/>
     </row>
     <row r="100" spans="1:10" ht="15">
-      <c r="A100" s="48"/>
-      <c r="B100" s="47"/>
-      <c r="C100" s="48"/>
-      <c r="D100" s="48"/>
+      <c r="A100" s="47"/>
+      <c r="B100" s="60"/>
+      <c r="C100" s="47"/>
+      <c r="D100" s="47"/>
       <c r="E100" s="5" t="s">
         <v>266</v>
       </c>
       <c r="F100" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="G100" s="63"/>
-      <c r="H100" s="69"/>
-      <c r="I100" s="61"/>
-      <c r="J100" s="68"/>
+      <c r="G100" s="51"/>
+      <c r="H100" s="53"/>
+      <c r="I100" s="56"/>
+      <c r="J100" s="58"/>
     </row>
     <row r="101" spans="1:10" ht="15">
       <c r="A101" s="8">
         <v>43</v>
       </c>
-      <c r="B101" s="47"/>
+      <c r="B101" s="60"/>
       <c r="C101" s="8" t="s">
         <v>341</v>
       </c>
@@ -4309,14 +4309,14 @@
       <c r="H101" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="I101" s="61"/>
-      <c r="J101" s="68"/>
+      <c r="I101" s="56"/>
+      <c r="J101" s="58"/>
     </row>
     <row r="102" spans="1:10" ht="15">
       <c r="A102" s="8">
         <v>44</v>
       </c>
-      <c r="B102" s="47"/>
+      <c r="B102" s="60"/>
       <c r="C102" s="8" t="s">
         <v>343</v>
       </c>
@@ -4335,74 +4335,74 @@
       <c r="H102" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="I102" s="63"/>
-      <c r="J102" s="69"/>
+      <c r="I102" s="51"/>
+      <c r="J102" s="53"/>
     </row>
     <row r="103" spans="1:10" ht="15">
       <c r="A103" s="8">
         <v>45</v>
       </c>
-      <c r="B103" s="47"/>
+      <c r="B103" s="60"/>
       <c r="C103" s="8" t="s">
         <v>345</v>
       </c>
       <c r="D103" s="35" t="s">
         <v>346</v>
       </c>
-      <c r="E103" s="51" t="s">
+      <c r="E103" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="F103" s="51" t="s">
+      <c r="F103" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="G103" s="66" t="s">
+      <c r="G103" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="H103" s="70"/>
-      <c r="I103" s="70"/>
-      <c r="J103" s="67"/>
+      <c r="H103" s="49"/>
+      <c r="I103" s="49"/>
+      <c r="J103" s="50"/>
     </row>
     <row r="104" spans="1:10" ht="15">
       <c r="A104" s="8">
         <v>46</v>
       </c>
-      <c r="B104" s="47"/>
+      <c r="B104" s="60"/>
       <c r="C104" s="8" t="s">
         <v>347</v>
       </c>
       <c r="D104" s="35" t="s">
         <v>348</v>
       </c>
-      <c r="E104" s="47"/>
-      <c r="F104" s="47"/>
-      <c r="G104" s="61"/>
-      <c r="H104" s="79"/>
-      <c r="I104" s="79"/>
-      <c r="J104" s="68"/>
+      <c r="E104" s="60"/>
+      <c r="F104" s="60"/>
+      <c r="G104" s="56"/>
+      <c r="H104" s="57"/>
+      <c r="I104" s="57"/>
+      <c r="J104" s="58"/>
     </row>
     <row r="105" spans="1:10" ht="15">
       <c r="A105" s="8">
         <v>47</v>
       </c>
-      <c r="B105" s="47"/>
+      <c r="B105" s="60"/>
       <c r="C105" s="8" t="s">
         <v>349</v>
       </c>
       <c r="D105" s="35" t="s">
         <v>350</v>
       </c>
-      <c r="E105" s="48"/>
-      <c r="F105" s="48"/>
-      <c r="G105" s="63"/>
-      <c r="H105" s="71"/>
-      <c r="I105" s="71"/>
-      <c r="J105" s="69"/>
+      <c r="E105" s="47"/>
+      <c r="F105" s="47"/>
+      <c r="G105" s="51"/>
+      <c r="H105" s="52"/>
+      <c r="I105" s="52"/>
+      <c r="J105" s="53"/>
     </row>
     <row r="106" spans="1:10" ht="15">
       <c r="A106" s="8">
         <v>48</v>
       </c>
-      <c r="B106" s="47"/>
+      <c r="B106" s="60"/>
       <c r="C106" s="8" t="s">
         <v>351</v>
       </c>
@@ -4421,14 +4421,14 @@
       <c r="H106" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="I106" s="66" t="s">
+      <c r="I106" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="J106" s="67"/>
+      <c r="J106" s="50"/>
     </row>
     <row r="107" spans="1:10" ht="15">
       <c r="A107" s="8"/>
-      <c r="B107" s="47"/>
+      <c r="B107" s="60"/>
       <c r="C107" s="8" t="s">
         <v>353</v>
       </c>
@@ -4447,16 +4447,16 @@
       <c r="H107" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="I107" s="61"/>
-      <c r="J107" s="68"/>
+      <c r="I107" s="56"/>
+      <c r="J107" s="58"/>
     </row>
     <row r="108" spans="1:10" ht="15">
       <c r="A108" s="8"/>
-      <c r="B108" s="47"/>
-      <c r="C108" s="46" t="s">
+      <c r="B108" s="60"/>
+      <c r="C108" s="61" t="s">
         <v>355</v>
       </c>
-      <c r="D108" s="53" t="s">
+      <c r="D108" s="65" t="s">
         <v>356</v>
       </c>
       <c r="E108" s="11" t="s">
@@ -4465,38 +4465,38 @@
       <c r="F108" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="G108" s="51" t="s">
+      <c r="G108" s="46" t="s">
         <v>193</v>
       </c>
-      <c r="H108" s="51" t="s">
+      <c r="H108" s="46" t="s">
         <v>194</v>
       </c>
-      <c r="I108" s="61"/>
-      <c r="J108" s="68"/>
+      <c r="I108" s="56"/>
+      <c r="J108" s="58"/>
     </row>
     <row r="109" spans="1:10" ht="15">
       <c r="A109" s="8">
         <v>49</v>
       </c>
-      <c r="B109" s="47"/>
-      <c r="C109" s="48"/>
-      <c r="D109" s="48"/>
+      <c r="B109" s="60"/>
+      <c r="C109" s="47"/>
+      <c r="D109" s="47"/>
       <c r="E109" s="5" t="s">
         <v>191</v>
       </c>
       <c r="F109" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="G109" s="48"/>
-      <c r="H109" s="48"/>
-      <c r="I109" s="61"/>
-      <c r="J109" s="68"/>
+      <c r="G109" s="47"/>
+      <c r="H109" s="47"/>
+      <c r="I109" s="56"/>
+      <c r="J109" s="58"/>
     </row>
     <row r="110" spans="1:10" ht="15">
       <c r="A110" s="8">
         <v>51</v>
       </c>
-      <c r="B110" s="47"/>
+      <c r="B110" s="60"/>
       <c r="C110" s="8" t="s">
         <v>357</v>
       </c>
@@ -4515,14 +4515,14 @@
       <c r="H110" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="I110" s="61"/>
-      <c r="J110" s="68"/>
+      <c r="I110" s="56"/>
+      <c r="J110" s="58"/>
     </row>
     <row r="111" spans="1:10" ht="15">
       <c r="A111" s="8">
         <v>52</v>
       </c>
-      <c r="B111" s="47"/>
+      <c r="B111" s="60"/>
       <c r="C111" s="8" t="s">
         <v>359</v>
       </c>
@@ -4541,12 +4541,12 @@
       <c r="H111" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="I111" s="61"/>
-      <c r="J111" s="68"/>
+      <c r="I111" s="56"/>
+      <c r="J111" s="58"/>
     </row>
     <row r="112" spans="1:10" ht="15">
       <c r="A112" s="8"/>
-      <c r="B112" s="47"/>
+      <c r="B112" s="60"/>
       <c r="C112" s="8" t="s">
         <v>361</v>
       </c>
@@ -4565,14 +4565,14 @@
       <c r="H112" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="I112" s="61"/>
-      <c r="J112" s="68"/>
+      <c r="I112" s="56"/>
+      <c r="J112" s="58"/>
     </row>
     <row r="113" spans="1:10" ht="30">
       <c r="A113" s="8">
         <v>54</v>
       </c>
-      <c r="B113" s="47"/>
+      <c r="B113" s="60"/>
       <c r="C113" s="8" t="s">
         <v>363</v>
       </c>
@@ -4591,12 +4591,12 @@
       <c r="H113" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="I113" s="61"/>
-      <c r="J113" s="68"/>
+      <c r="I113" s="56"/>
+      <c r="J113" s="58"/>
     </row>
     <row r="114" spans="1:10" ht="30">
       <c r="A114" s="8"/>
-      <c r="B114" s="47"/>
+      <c r="B114" s="60"/>
       <c r="C114" s="8" t="s">
         <v>365</v>
       </c>
@@ -4615,12 +4615,12 @@
       <c r="H114" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="I114" s="61"/>
-      <c r="J114" s="68"/>
+      <c r="I114" s="56"/>
+      <c r="J114" s="58"/>
     </row>
     <row r="115" spans="1:10" ht="30">
       <c r="A115" s="8"/>
-      <c r="B115" s="47"/>
+      <c r="B115" s="60"/>
       <c r="C115" s="8" t="s">
         <v>367</v>
       </c>
@@ -4639,14 +4639,14 @@
       <c r="H115" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="I115" s="61"/>
-      <c r="J115" s="68"/>
+      <c r="I115" s="56"/>
+      <c r="J115" s="58"/>
     </row>
     <row r="116" spans="1:10" ht="30">
       <c r="A116" s="8">
         <v>57</v>
       </c>
-      <c r="B116" s="47"/>
+      <c r="B116" s="60"/>
       <c r="C116" s="8" t="s">
         <v>369</v>
       </c>
@@ -4665,18 +4665,18 @@
       <c r="H116" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="I116" s="61"/>
-      <c r="J116" s="68"/>
+      <c r="I116" s="56"/>
+      <c r="J116" s="58"/>
     </row>
     <row r="117" spans="1:10" ht="30">
       <c r="A117" s="8">
         <v>58</v>
       </c>
-      <c r="B117" s="47"/>
-      <c r="C117" s="46" t="s">
+      <c r="B117" s="60"/>
+      <c r="C117" s="61" t="s">
         <v>371</v>
       </c>
-      <c r="D117" s="53" t="s">
+      <c r="D117" s="65" t="s">
         <v>372</v>
       </c>
       <c r="E117" s="11" t="s">
@@ -4691,14 +4691,14 @@
       <c r="H117" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="I117" s="61"/>
-      <c r="J117" s="68"/>
+      <c r="I117" s="56"/>
+      <c r="J117" s="58"/>
     </row>
     <row r="118" spans="1:10" ht="15">
       <c r="A118" s="8"/>
-      <c r="B118" s="47"/>
-      <c r="C118" s="48"/>
-      <c r="D118" s="48"/>
+      <c r="B118" s="60"/>
+      <c r="C118" s="47"/>
+      <c r="D118" s="47"/>
       <c r="E118" s="11" t="s">
         <v>250</v>
       </c>
@@ -4711,24 +4711,24 @@
       <c r="H118" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="I118" s="61"/>
-      <c r="J118" s="68"/>
+      <c r="I118" s="56"/>
+      <c r="J118" s="58"/>
     </row>
     <row r="119" spans="1:10" ht="15">
       <c r="A119" s="8">
         <v>59</v>
       </c>
-      <c r="B119" s="47"/>
-      <c r="C119" s="46" t="s">
+      <c r="B119" s="60"/>
+      <c r="C119" s="61" t="s">
         <v>373</v>
       </c>
-      <c r="D119" s="53" t="s">
+      <c r="D119" s="65" t="s">
         <v>374</v>
       </c>
-      <c r="E119" s="51" t="s">
+      <c r="E119" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="F119" s="51" t="s">
+      <c r="F119" s="46" t="s">
         <v>64</v>
       </c>
       <c r="G119" s="5" t="s">
@@ -4737,30 +4737,30 @@
       <c r="H119" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="I119" s="61"/>
-      <c r="J119" s="68"/>
+      <c r="I119" s="56"/>
+      <c r="J119" s="58"/>
     </row>
     <row r="120" spans="1:10" ht="15">
       <c r="A120" s="8"/>
-      <c r="B120" s="47"/>
-      <c r="C120" s="48"/>
-      <c r="D120" s="48"/>
-      <c r="E120" s="48"/>
-      <c r="F120" s="48"/>
+      <c r="B120" s="60"/>
+      <c r="C120" s="47"/>
+      <c r="D120" s="47"/>
+      <c r="E120" s="47"/>
+      <c r="F120" s="47"/>
       <c r="G120" s="5" t="s">
         <v>167</v>
       </c>
       <c r="H120" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="I120" s="61"/>
-      <c r="J120" s="68"/>
+      <c r="I120" s="56"/>
+      <c r="J120" s="58"/>
     </row>
     <row r="121" spans="1:10" ht="30">
       <c r="A121" s="8">
         <v>60</v>
       </c>
-      <c r="B121" s="47"/>
+      <c r="B121" s="60"/>
       <c r="C121" s="8" t="s">
         <v>375</v>
       </c>
@@ -4779,14 +4779,14 @@
       <c r="H121" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="I121" s="61"/>
-      <c r="J121" s="68"/>
+      <c r="I121" s="56"/>
+      <c r="J121" s="58"/>
     </row>
     <row r="122" spans="1:10" ht="30">
       <c r="A122" s="8">
         <v>61</v>
       </c>
-      <c r="B122" s="48"/>
+      <c r="B122" s="47"/>
       <c r="C122" s="8" t="s">
         <v>377</v>
       </c>
@@ -4805,8 +4805,8 @@
       <c r="H122" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="I122" s="63"/>
-      <c r="J122" s="69"/>
+      <c r="I122" s="51"/>
+      <c r="J122" s="53"/>
     </row>
     <row r="123" spans="1:10" ht="14" hidden="1">
       <c r="A123" s="38"/>
@@ -15874,15 +15874,151 @@
     </row>
   </sheetData>
   <mergeCells count="178">
-    <mergeCell ref="G108:G109"/>
-    <mergeCell ref="H108:H109"/>
-    <mergeCell ref="G84:J85"/>
-    <mergeCell ref="I86:J86"/>
-    <mergeCell ref="G87:J92"/>
-    <mergeCell ref="I93:J102"/>
-    <mergeCell ref="G96:H100"/>
-    <mergeCell ref="G103:J105"/>
-    <mergeCell ref="I106:J122"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="D26:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="F32:F33"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="D29:D31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="E34:E38"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="A34:A38"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="C34:C38"/>
+    <mergeCell ref="D34:D38"/>
+    <mergeCell ref="F34:F38"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="D39:D41"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="C39:C41"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="E42:E45"/>
+    <mergeCell ref="F42:F45"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="E47:E49"/>
+    <mergeCell ref="F47:F49"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="I4:J55"/>
+    <mergeCell ref="G56:J57"/>
+    <mergeCell ref="G58:J58"/>
+    <mergeCell ref="G59:J59"/>
+    <mergeCell ref="I60:J62"/>
+    <mergeCell ref="G63:H64"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:J1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="A4:A9"/>
+    <mergeCell ref="B4:B9"/>
+    <mergeCell ref="C4:C9"/>
+    <mergeCell ref="D4:D9"/>
+    <mergeCell ref="E5:E10"/>
+    <mergeCell ref="F5:F10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="A13:A18"/>
+    <mergeCell ref="C13:C18"/>
+    <mergeCell ref="D13:D18"/>
+    <mergeCell ref="E13:F18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B13:B18"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="E58:E59"/>
+    <mergeCell ref="F58:F59"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="B50:B52"/>
+    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="D50:D52"/>
+    <mergeCell ref="E50:E52"/>
+    <mergeCell ref="F50:F52"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="C60:C62"/>
+    <mergeCell ref="D60:D62"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="D53:D54"/>
+    <mergeCell ref="A63:A64"/>
+    <mergeCell ref="B63:B64"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="D63:D64"/>
+    <mergeCell ref="E63:E64"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="D65:D66"/>
+    <mergeCell ref="A67:A68"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A71:A72"/>
+    <mergeCell ref="A73:A74"/>
+    <mergeCell ref="B93:B122"/>
+    <mergeCell ref="A96:A100"/>
+    <mergeCell ref="C108:C109"/>
+    <mergeCell ref="C117:C118"/>
+    <mergeCell ref="D117:D118"/>
+    <mergeCell ref="C119:C120"/>
+    <mergeCell ref="D119:D120"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="B87:B90"/>
+    <mergeCell ref="A76:A77"/>
+    <mergeCell ref="B76:B77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="E119:E120"/>
+    <mergeCell ref="F119:F120"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="C69:C70"/>
+    <mergeCell ref="C96:C100"/>
+    <mergeCell ref="D96:D100"/>
+    <mergeCell ref="E103:E105"/>
+    <mergeCell ref="F103:F105"/>
+    <mergeCell ref="D108:D109"/>
+    <mergeCell ref="D67:D68"/>
+    <mergeCell ref="E87:E90"/>
+    <mergeCell ref="F87:F90"/>
+    <mergeCell ref="C76:C77"/>
     <mergeCell ref="G67:H74"/>
     <mergeCell ref="I67:J81"/>
     <mergeCell ref="G75:H75"/>
@@ -15907,151 +16043,15 @@
     <mergeCell ref="B71:B74"/>
     <mergeCell ref="C71:C72"/>
     <mergeCell ref="C73:C74"/>
-    <mergeCell ref="E119:E120"/>
-    <mergeCell ref="F119:F120"/>
-    <mergeCell ref="C67:C68"/>
-    <mergeCell ref="C69:C70"/>
-    <mergeCell ref="C96:C100"/>
-    <mergeCell ref="D96:D100"/>
-    <mergeCell ref="E103:E105"/>
-    <mergeCell ref="F103:F105"/>
-    <mergeCell ref="D108:D109"/>
-    <mergeCell ref="D67:D68"/>
-    <mergeCell ref="E87:E90"/>
-    <mergeCell ref="F87:F90"/>
-    <mergeCell ref="C76:C77"/>
-    <mergeCell ref="A71:A72"/>
-    <mergeCell ref="A73:A74"/>
-    <mergeCell ref="B93:B122"/>
-    <mergeCell ref="A96:A100"/>
-    <mergeCell ref="C108:C109"/>
-    <mergeCell ref="C117:C118"/>
-    <mergeCell ref="D117:D118"/>
-    <mergeCell ref="C119:C120"/>
-    <mergeCell ref="D119:D120"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="B87:B90"/>
-    <mergeCell ref="A76:A77"/>
-    <mergeCell ref="B76:B77"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A63:A64"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="C63:C64"/>
-    <mergeCell ref="D63:D64"/>
-    <mergeCell ref="E63:E64"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="D65:D66"/>
-    <mergeCell ref="A67:A68"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="C60:C62"/>
-    <mergeCell ref="D60:D62"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A56:A57"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="A60:A62"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="D53:D54"/>
-    <mergeCell ref="E53:E54"/>
-    <mergeCell ref="E58:E59"/>
-    <mergeCell ref="F58:F59"/>
-    <mergeCell ref="A50:A52"/>
-    <mergeCell ref="B50:B52"/>
-    <mergeCell ref="C50:C52"/>
-    <mergeCell ref="D50:D52"/>
-    <mergeCell ref="E50:E52"/>
-    <mergeCell ref="F50:F52"/>
-    <mergeCell ref="F53:F54"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="D19:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="A13:A18"/>
-    <mergeCell ref="C13:C18"/>
-    <mergeCell ref="D13:D18"/>
-    <mergeCell ref="E13:F18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="I4:J55"/>
-    <mergeCell ref="G56:J57"/>
-    <mergeCell ref="G58:J58"/>
-    <mergeCell ref="G59:J59"/>
-    <mergeCell ref="I60:J62"/>
-    <mergeCell ref="G63:H64"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:J1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="A4:A9"/>
-    <mergeCell ref="B4:B9"/>
-    <mergeCell ref="C4:C9"/>
-    <mergeCell ref="D4:D9"/>
-    <mergeCell ref="E5:E10"/>
-    <mergeCell ref="F5:F10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="E42:E45"/>
-    <mergeCell ref="F42:F45"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="D46:D49"/>
-    <mergeCell ref="E47:E49"/>
-    <mergeCell ref="F47:F49"/>
-    <mergeCell ref="E34:E38"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="A34:A38"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="C34:C38"/>
-    <mergeCell ref="D34:D38"/>
-    <mergeCell ref="F34:F38"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="D39:D41"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="C39:C41"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="F32:F33"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="D29:D31"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="B13:B18"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="E23:E25"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="D26:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="G108:G109"/>
+    <mergeCell ref="H108:H109"/>
+    <mergeCell ref="G84:J85"/>
+    <mergeCell ref="I86:J86"/>
+    <mergeCell ref="G87:J92"/>
+    <mergeCell ref="I93:J102"/>
+    <mergeCell ref="G96:H100"/>
+    <mergeCell ref="G103:J105"/>
+    <mergeCell ref="I106:J122"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>